<commit_message>
Update infant unit tests
</commit_message>
<xml_diff>
--- a/data/tier_app/country_costs.xlsx
+++ b/data/tier_app/country_costs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/tier_app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{A44B6979-C974-2F43-A899-180A4F7BAE89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3C22998-F053-A14B-8830-DA286B7E3C1C}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{A44B6979-C974-2F43-A899-180A4F7BAE89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C779809C-0E00-3141-AE3A-53E70C3E543B}"/>
   <bookViews>
-    <workbookView xWindow="440" yWindow="6620" windowWidth="27640" windowHeight="15280" xr2:uid="{A508B7DC-02AE-4845-B676-FDD92F1561DC}"/>
+    <workbookView xWindow="440" yWindow="1140" windowWidth="27640" windowHeight="15280" xr2:uid="{A508B7DC-02AE-4845-B676-FDD92F1561DC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Zambia</t>
   </si>
@@ -83,17 +83,29 @@
     <t>Zimbabwe</t>
   </si>
   <si>
-    <t>art_cost_standard</t>
-  </si>
-  <si>
     <t>country</t>
+  </si>
+  <si>
+    <t>Cost of treatment</t>
+  </si>
+  <si>
+    <t>Botswana</t>
+  </si>
+  <si>
+    <t>C'ote d'ivoire</t>
+  </si>
+  <si>
+    <t>Nigeria</t>
+  </si>
+  <si>
+    <t>Tanzania</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -115,12 +127,6 @@
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -183,8 +189,8 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -520,7 +526,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F954A092-A5F1-D044-85EF-FAF8818A0818}">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
@@ -529,10 +535,10 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>16</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -607,7 +613,7 @@
         <v>101.9</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="34" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" ht="17" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
@@ -631,7 +637,7 @@
         <v>113.46</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="34" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>12</v>
       </c>
@@ -655,9 +661,49 @@
         <v>130.18</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
+    <row r="17" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="4">
+        <v>221.82</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="4">
+        <v>144.28</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="4">
+        <v>151.94</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="4">
+        <v>120.74</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Indiviudal country ART costs
</commit_message>
<xml_diff>
--- a/data/tier_app/country_costs.xlsx
+++ b/data/tier_app/country_costs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/tier_app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{A44B6979-C974-2F43-A899-180A4F7BAE89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C779809C-0E00-3141-AE3A-53E70C3E543B}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{A44B6979-C974-2F43-A899-180A4F7BAE89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E746C9AC-21AC-9149-BBB5-DBFAF06F59FF}"/>
   <bookViews>
-    <workbookView xWindow="440" yWindow="1140" windowWidth="27640" windowHeight="15280" xr2:uid="{A508B7DC-02AE-4845-B676-FDD92F1561DC}"/>
+    <workbookView xWindow="1860" yWindow="600" windowWidth="27640" windowHeight="15280" xr2:uid="{A508B7DC-02AE-4845-B676-FDD92F1561DC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -83,29 +83,29 @@
     <t>Zimbabwe</t>
   </si>
   <si>
+    <t>art_cost_standard</t>
+  </si>
+  <si>
     <t>country</t>
   </si>
   <si>
-    <t>Cost of treatment</t>
-  </si>
-  <si>
     <t>Botswana</t>
   </si>
   <si>
-    <t>C'ote d'ivoire</t>
-  </si>
-  <si>
     <t>Nigeria</t>
   </si>
   <si>
-    <t>Tanzania</t>
+    <t>United Republic of Tanzania</t>
+  </si>
+  <si>
+    <t>Côte d'Ivoire</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -127,6 +127,12 @@
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -189,8 +195,8 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -535,10 +541,10 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>15</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -669,9 +675,9 @@
         <v>221.82</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B18" s="4">
         <v>144.28</v>
@@ -679,15 +685,15 @@
     </row>
     <row r="19" spans="1:2" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B19" s="4">
         <v>151.94</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" ht="34" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B20" s="4">
         <v>120.74</v>

</xml_diff>

<commit_message>
Adjusting oral prep to annual cost
</commit_message>
<xml_diff>
--- a/data/tier_app/country_costs.xlsx
+++ b/data/tier_app/country_costs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/tier_app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="58" documentId="8_{A44B6979-C974-2F43-A899-180A4F7BAE89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{973E1F22-1C3A-CF44-9E4C-A28B3EC62C24}"/>
+  <xr:revisionPtr revIDLastSave="59" documentId="8_{A44B6979-C974-2F43-A899-180A4F7BAE89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{20931531-4C3C-634E-B56E-47E6B36AC622}"/>
   <bookViews>
-    <workbookView xWindow="1160" yWindow="600" windowWidth="27640" windowHeight="15280" xr2:uid="{A508B7DC-02AE-4845-B676-FDD92F1561DC}"/>
+    <workbookView xWindow="-32700" yWindow="560" windowWidth="27640" windowHeight="15280" xr2:uid="{A508B7DC-02AE-4845-B676-FDD92F1561DC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -264,6 +264,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -683,17 +687,17 @@
       <c r="K2" s="1">
         <v>1.745331695</v>
       </c>
-      <c r="L2">
-        <v>47.811897250000001</v>
-      </c>
-      <c r="M2">
-        <v>48.92286</v>
-      </c>
-      <c r="N2">
-        <v>46.049460000000003</v>
-      </c>
-      <c r="O2">
-        <v>47.811897250000001</v>
+      <c r="L2" s="1">
+        <v>90.724662719999998</v>
+      </c>
+      <c r="M2" s="1">
+        <v>92.133444420000004</v>
+      </c>
+      <c r="N2" s="1">
+        <v>88.217350800000006</v>
+      </c>
+      <c r="O2" s="1">
+        <v>90.38165832</v>
       </c>
       <c r="P2">
         <v>40.768770000000004</v>
@@ -742,17 +746,17 @@
       <c r="K3" s="1">
         <v>2.8419164619999999</v>
       </c>
-      <c r="L3">
-        <v>54.87190983</v>
-      </c>
-      <c r="M3">
-        <v>56.146920000000001</v>
-      </c>
-      <c r="N3">
-        <v>52.849220000000003</v>
-      </c>
-      <c r="O3">
-        <v>54.87190983</v>
+      <c r="L3" s="1">
+        <v>104.12127099999999</v>
+      </c>
+      <c r="M3" s="1">
+        <v>105.7380766</v>
+      </c>
+      <c r="N3" s="1">
+        <v>101.2437238</v>
+      </c>
+      <c r="O3" s="1">
+        <v>103.7276178</v>
       </c>
       <c r="P3">
         <v>44.06174</v>
@@ -801,17 +805,17 @@
       <c r="K4" s="1">
         <v>3.5922113019999999</v>
       </c>
-      <c r="L4">
-        <v>59.702444749999998</v>
-      </c>
-      <c r="M4">
-        <v>61.089700000000001</v>
-      </c>
-      <c r="N4">
-        <v>57.5017</v>
-      </c>
-      <c r="O4">
-        <v>59.702444749999998</v>
+      <c r="L4" s="1">
+        <v>113.28737150000001</v>
+      </c>
+      <c r="M4" s="1">
+        <v>115.0465092</v>
+      </c>
+      <c r="N4" s="1">
+        <v>110.15650530000001</v>
+      </c>
+      <c r="O4" s="1">
+        <v>112.8590638</v>
       </c>
       <c r="P4">
         <v>46.314819999999997</v>
@@ -860,17 +864,17 @@
       <c r="K5" s="1">
         <v>1.743341523</v>
       </c>
-      <c r="L5">
-        <v>47.79908416</v>
-      </c>
-      <c r="M5">
-        <v>48.909750000000003</v>
-      </c>
-      <c r="N5">
-        <v>46.037120000000002</v>
-      </c>
-      <c r="O5">
-        <v>47.79908416</v>
+      <c r="L5" s="1">
+        <v>90.700349459999998</v>
+      </c>
+      <c r="M5" s="1">
+        <v>92.108753620000002</v>
+      </c>
+      <c r="N5" s="1">
+        <v>88.193709470000002</v>
+      </c>
+      <c r="O5" s="1">
+        <v>90.357436980000003</v>
       </c>
       <c r="P5">
         <v>40.762790000000003</v>
@@ -919,17 +923,17 @@
       <c r="K6" s="1">
         <v>2.5533415229999998</v>
       </c>
-      <c r="L6">
-        <v>53.014011789999998</v>
-      </c>
-      <c r="M6">
-        <v>54.245849999999997</v>
-      </c>
-      <c r="N6">
-        <v>51.059809999999999</v>
-      </c>
-      <c r="O6">
-        <v>53.014011789999998</v>
+      <c r="L6" s="1">
+        <v>100.5958478</v>
+      </c>
+      <c r="M6" s="1">
+        <v>102.1579102</v>
+      </c>
+      <c r="N6" s="1">
+        <v>97.815730889999998</v>
+      </c>
+      <c r="O6" s="1">
+        <v>100.21552320000001</v>
       </c>
       <c r="P6">
         <v>43.195169999999997</v>
@@ -978,17 +982,17 @@
       <c r="K7" s="1">
         <v>2.3782063880000002</v>
       </c>
-      <c r="L7">
-        <v>51.886459870000003</v>
-      </c>
-      <c r="M7">
-        <v>53.092100000000002</v>
-      </c>
-      <c r="N7">
-        <v>49.973820000000003</v>
-      </c>
-      <c r="O7">
-        <v>51.886459870000003</v>
+      <c r="L7" s="1">
+        <v>98.456280579999998</v>
+      </c>
+      <c r="M7" s="1">
+        <v>99.98511963</v>
+      </c>
+      <c r="N7" s="1">
+        <v>95.735293830000003</v>
+      </c>
+      <c r="O7" s="1">
+        <v>98.084045119999999</v>
       </c>
       <c r="P7">
         <v>42.669249999999998</v>
@@ -1037,17 +1041,17 @@
       <c r="K8" s="1">
         <v>1.424914005</v>
       </c>
-      <c r="L8">
-        <v>45.748989770000001</v>
-      </c>
-      <c r="M8">
-        <v>46.812019999999997</v>
-      </c>
-      <c r="N8">
-        <v>44.06259</v>
-      </c>
-      <c r="O8">
-        <v>45.748989770000001</v>
+      <c r="L8" s="1">
+        <v>86.810227260000005</v>
+      </c>
+      <c r="M8" s="1">
+        <v>88.158225220000006</v>
+      </c>
+      <c r="N8" s="1">
+        <v>84.411096630000003</v>
+      </c>
+      <c r="O8" s="1">
+        <v>86.482022240000006</v>
       </c>
       <c r="P8">
         <v>39.806570000000001</v>
@@ -1096,17 +1100,17 @@
       <c r="K9" s="1">
         <v>1.2099754300000001</v>
       </c>
-      <c r="L9">
-        <v>44.365176050000002</v>
-      </c>
-      <c r="M9">
-        <v>45.396050000000002</v>
-      </c>
-      <c r="N9">
-        <v>42.729790000000001</v>
-      </c>
-      <c r="O9">
-        <v>44.365176050000002</v>
+      <c r="L9" s="1">
+        <v>84.184394780000005</v>
+      </c>
+      <c r="M9" s="1">
+        <v>85.491618540000005</v>
+      </c>
+      <c r="N9" s="1">
+        <v>81.857832959999996</v>
+      </c>
+      <c r="O9" s="1">
+        <v>83.866117290000005</v>
       </c>
       <c r="P9">
         <v>39.16113</v>
@@ -1155,17 +1159,17 @@
       <c r="K10" s="1">
         <v>1.1562407859999999</v>
       </c>
-      <c r="L10">
-        <v>44.019222620000001</v>
-      </c>
-      <c r="M10">
-        <v>45.042059999999999</v>
-      </c>
-      <c r="N10">
-        <v>42.396590000000003</v>
-      </c>
-      <c r="O10">
-        <v>44.019222620000001</v>
+      <c r="L10" s="1">
+        <v>83.527936659999995</v>
+      </c>
+      <c r="M10" s="1">
+        <v>84.824966869999997</v>
+      </c>
+      <c r="N10" s="1">
+        <v>81.219517039999999</v>
+      </c>
+      <c r="O10" s="1">
+        <v>83.212141059999993</v>
       </c>
       <c r="P10">
         <v>38.999769999999998</v>
@@ -1214,17 +1218,17 @@
       <c r="K11" s="1">
         <v>1.154250614</v>
       </c>
-      <c r="L11">
-        <v>44.006409529999999</v>
-      </c>
-      <c r="M11">
-        <v>45.028950000000002</v>
-      </c>
-      <c r="N11">
-        <v>42.384250000000002</v>
-      </c>
-      <c r="O11">
-        <v>44.006409529999999</v>
+      <c r="L11" s="1">
+        <v>83.503623399999995</v>
+      </c>
+      <c r="M11" s="1">
+        <v>84.800276069999995</v>
+      </c>
+      <c r="N11" s="1">
+        <v>81.195875709999996</v>
+      </c>
+      <c r="O11" s="1">
+        <v>83.187919719999996</v>
       </c>
       <c r="P11">
         <v>38.993789999999997</v>
@@ -1273,17 +1277,17 @@
       <c r="K12" s="1">
         <v>3.3474201469999998</v>
       </c>
-      <c r="L12">
-        <v>58.126434690000004</v>
-      </c>
-      <c r="M12">
-        <v>59.477069999999998</v>
-      </c>
-      <c r="N12">
-        <v>55.983780000000003</v>
-      </c>
-      <c r="O12">
-        <v>58.126434690000004</v>
+      <c r="L12" s="1">
+        <v>110.29684</v>
+      </c>
+      <c r="M12" s="1">
+        <v>112.0095405</v>
+      </c>
+      <c r="N12" s="1">
+        <v>107.2486217</v>
+      </c>
+      <c r="O12" s="1">
+        <v>109.87983869999999</v>
       </c>
       <c r="P12">
         <v>45.579729999999998</v>
@@ -1332,17 +1336,17 @@
       <c r="K13" s="1">
         <v>1.673685504</v>
       </c>
-      <c r="L13">
-        <v>47.350626009999999</v>
-      </c>
-      <c r="M13">
-        <v>48.450870000000002</v>
-      </c>
-      <c r="N13">
-        <v>45.60519</v>
-      </c>
-      <c r="O13">
-        <v>47.350626009999999</v>
+      <c r="L13" s="1">
+        <v>89.849385229999996</v>
+      </c>
+      <c r="M13" s="1">
+        <v>91.244575530000006</v>
+      </c>
+      <c r="N13" s="1">
+        <v>87.366262910000003</v>
+      </c>
+      <c r="O13" s="1">
+        <v>89.50969001</v>
       </c>
       <c r="P13">
         <v>40.553620000000002</v>
@@ -1391,17 +1395,17 @@
       <c r="K14" s="1">
         <v>3.8131740000000001</v>
       </c>
-      <c r="L14">
-        <v>62.585389999999997</v>
-      </c>
-      <c r="M14">
-        <v>64.039630000000002</v>
-      </c>
-      <c r="N14">
-        <v>60.278370000000002</v>
-      </c>
-      <c r="O14">
-        <v>62.585389999999997</v>
+      <c r="L14" s="1">
+        <v>118.7578558</v>
+      </c>
+      <c r="M14" s="1">
+        <v>120.6019397</v>
+      </c>
+      <c r="N14" s="1">
+        <v>115.4758046</v>
+      </c>
+      <c r="O14" s="1">
+        <v>118.30886580000001</v>
       </c>
       <c r="P14">
         <v>47.659500000000001</v>
@@ -1450,17 +1454,17 @@
       <c r="K15" s="1">
         <v>1.6219410320000001</v>
       </c>
-      <c r="L15">
-        <v>47.017485669999999</v>
-      </c>
-      <c r="M15">
-        <v>48.109990000000003</v>
-      </c>
-      <c r="N15">
-        <v>45.284329999999997</v>
-      </c>
-      <c r="O15">
-        <v>47.017485669999999</v>
+      <c r="L15" s="1">
+        <v>89.217240369999999</v>
+      </c>
+      <c r="M15" s="1">
+        <v>90.602614669999994</v>
+      </c>
+      <c r="N15" s="1">
+        <v>86.751588319999996</v>
+      </c>
+      <c r="O15" s="1">
+        <v>88.879935110000005</v>
       </c>
       <c r="P15">
         <v>40.398229999999998</v>
@@ -1509,17 +1513,17 @@
       <c r="K16" s="1">
         <v>2.425970516</v>
       </c>
-      <c r="L16">
-        <v>52.19397403</v>
-      </c>
-      <c r="M16">
-        <v>53.406759999999998</v>
-      </c>
-      <c r="N16">
-        <v>50.27</v>
-      </c>
-      <c r="O16">
-        <v>52.19397403</v>
+      <c r="L16" s="1">
+        <v>99.039798910000002</v>
+      </c>
+      <c r="M16" s="1">
+        <v>100.5776989</v>
+      </c>
+      <c r="N16" s="1">
+        <v>96.302685749999995</v>
+      </c>
+      <c r="O16" s="1">
+        <v>98.665357330000006</v>
       </c>
       <c r="P16">
         <v>42.81268</v>
@@ -1568,17 +1572,17 @@
       <c r="K17" s="1">
         <v>5.1863390660000004</v>
       </c>
-      <c r="L17">
-        <v>69.965729830000001</v>
-      </c>
-      <c r="M17">
-        <v>71.591459999999998</v>
-      </c>
-      <c r="N17">
-        <v>67.386660000000006</v>
-      </c>
-      <c r="O17">
-        <v>69.965729830000001</v>
+      <c r="L17" s="1">
+        <v>132.76229570000001</v>
+      </c>
+      <c r="M17" s="1">
+        <v>134.82384200000001</v>
+      </c>
+      <c r="N17" s="1">
+        <v>129.09321080000001</v>
+      </c>
+      <c r="O17" s="1">
+        <v>132.26035880000001</v>
       </c>
       <c r="P17">
         <v>51.101880000000001</v>
@@ -1627,17 +1631,17 @@
       <c r="K18" s="1">
         <v>2.525479115</v>
       </c>
-      <c r="L18">
-        <v>52.834628530000003</v>
-      </c>
-      <c r="M18">
-        <v>54.0623</v>
-      </c>
-      <c r="N18">
-        <v>50.887039999999999</v>
-      </c>
-      <c r="O18">
-        <v>52.834628530000003</v>
+      <c r="L18" s="1">
+        <v>100.2554621</v>
+      </c>
+      <c r="M18" s="1">
+        <v>101.81223900000001</v>
+      </c>
+      <c r="N18" s="1">
+        <v>97.484752270000001</v>
+      </c>
+      <c r="O18" s="1">
+        <v>99.87642443</v>
       </c>
       <c r="P18">
         <v>43.111499999999999</v>
@@ -1686,17 +1690,17 @@
       <c r="K19" s="1">
         <v>2.788181818</v>
       </c>
-      <c r="L19">
-        <v>54.525956399999998</v>
-      </c>
-      <c r="M19">
-        <v>55.792929999999998</v>
-      </c>
-      <c r="N19">
-        <v>52.516019999999997</v>
-      </c>
-      <c r="O19">
-        <v>54.525956399999998</v>
+      <c r="L19" s="1">
+        <v>103.4648129</v>
+      </c>
+      <c r="M19" s="1">
+        <v>105.0714249</v>
+      </c>
+      <c r="N19" s="1">
+        <v>100.6054079</v>
+      </c>
+      <c r="O19" s="1">
+        <v>103.0736416</v>
       </c>
       <c r="P19">
         <v>43.900379999999998</v>
@@ -1745,17 +1749,17 @@
       <c r="K20" s="1">
         <v>1.7174692869999999</v>
       </c>
-      <c r="L20">
-        <v>47.63251399</v>
-      </c>
-      <c r="M20">
-        <v>48.739310000000003</v>
-      </c>
-      <c r="N20">
-        <v>45.876690000000004</v>
-      </c>
-      <c r="O20">
-        <v>47.63251399</v>
+      <c r="L20" s="1">
+        <v>90.384277030000007</v>
+      </c>
+      <c r="M20" s="1">
+        <v>91.787773189999996</v>
+      </c>
+      <c r="N20" s="1">
+        <v>87.886372179999995</v>
+      </c>
+      <c r="O20" s="1">
+        <v>90.042559530000005</v>
       </c>
       <c r="P20">
         <v>40.685099999999998</v>

</xml_diff>